<commit_message>
updated RPom_membrane_lipid_comp.xlsx uploaded for lipid biomass coefficient review
</commit_message>
<xml_diff>
--- a/model_building/reactions/corrections/RPom_membrane_lipid_comp.xlsx
+++ b/model_building/reactions/corrections/RPom_membrane_lipid_comp.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/acheron/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37ADEBA-41AC-9844-A539-220B2D53D450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3FE3571-09B8-2D48-8845-B281D66335F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{D094A239-479A-424F-BFF7-7679225784C9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -220,7 +220,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -268,8 +268,16 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -279,6 +287,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -295,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -303,8 +317,11 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -640,7 +657,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAB04D88-6EB3-3440-9E55-06BDA8EC0F88}">
   <dimension ref="A1:K49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -702,12 +719,12 @@
         <v>0.46921840821833111</v>
       </c>
       <c r="G2" s="2">
-        <f>1/1000*D2/E2</f>
-        <v>1.2307627491803279</v>
+        <f>(D2/1000)*E2</f>
+        <v>0.48554762821834663</v>
       </c>
       <c r="H2" s="2">
-        <f>1/1000*D2/F2</f>
-        <v>1.6475099579646018</v>
+        <f>(D2/1000)*F2</f>
+        <v>0.36272553672591512</v>
       </c>
       <c r="J2" s="6"/>
     </row>
@@ -736,12 +753,12 @@
         <v>5.8950362797503639E-2</v>
       </c>
       <c r="G3" s="2">
-        <f t="shared" ref="G3:G8" si="2">1/1000*D3/E3</f>
-        <v>16.320984282608695</v>
+        <f t="shared" ref="G3:G9" si="2">(D3/1000)*E3</f>
+        <v>3.3919977908067271E-2</v>
       </c>
       <c r="H3" s="2">
-        <f t="shared" ref="H3:H9" si="3">1/1000*D3/F3</f>
-        <v>12.621601711864411</v>
+        <f t="shared" ref="H3:H9" si="3">(D3/1000)*F3</f>
+        <v>4.3861899538756993E-2</v>
       </c>
       <c r="J3" s="6"/>
     </row>
@@ -771,11 +788,11 @@
       </c>
       <c r="G4" s="2">
         <f t="shared" si="2"/>
-        <v>6.0061222159999996</v>
+        <v>9.5681986639247596E-2</v>
       </c>
       <c r="H4" s="2">
         <f t="shared" si="3"/>
-        <v>3.8584171036269437</v>
+        <v>0.14894131199159322</v>
       </c>
       <c r="J4" s="6"/>
     </row>
@@ -805,11 +822,11 @@
       </c>
       <c r="G5" s="2">
         <f t="shared" si="2"/>
-        <v>75.076527699999986</v>
+        <v>7.940451119238431E-3</v>
       </c>
       <c r="H5" s="2">
         <f t="shared" si="3"/>
-        <v>46.542156312499962</v>
+        <v>1.28086351307254E-2</v>
       </c>
       <c r="J5" s="6"/>
     </row>
@@ -837,11 +854,11 @@
       </c>
       <c r="G6" s="2">
         <f t="shared" si="2"/>
-        <v>150.1530554</v>
+        <v>1.5318460447725265E-3</v>
       </c>
       <c r="H6" s="2">
         <f t="shared" si="3"/>
-        <v>248.22483366666665</v>
+        <v>9.2662511090197807E-4</v>
       </c>
       <c r="J6" s="6"/>
     </row>
@@ -871,11 +888,11 @@
       </c>
       <c r="G7" s="2">
         <f t="shared" si="2"/>
-        <v>11.205451895522391</v>
+        <v>4.1032442605882527E-2</v>
       </c>
       <c r="H7" s="2">
         <f t="shared" si="3"/>
-        <v>28.641326961538486</v>
+        <v>1.6053273732513623E-2</v>
       </c>
       <c r="J7" s="6"/>
     </row>
@@ -904,11 +921,11 @@
       </c>
       <c r="G8" s="2">
         <f t="shared" si="2"/>
-        <v>5.4800385182481763</v>
+        <v>8.7143818973312748E-2</v>
       </c>
       <c r="H8" s="2">
         <f t="shared" si="3"/>
-        <v>3.0645041193415636</v>
+        <v>0.15583320041469104</v>
       </c>
       <c r="J8" s="6"/>
     </row>
@@ -935,13 +952,17 @@
         <v>7.6602918353451191E-3</v>
       </c>
       <c r="G9" s="2">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="H9" s="2">
         <f t="shared" si="3"/>
-        <v>93.084312624999995</v>
+        <v>5.4621940740683435E-3</v>
       </c>
       <c r="J9" s="6"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J10" s="6"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -956,7 +977,7 @@
         <v>99.999999999999986</v>
       </c>
       <c r="E11">
-        <f>SUM(E2:E9)</f>
+        <f>SUM(E2:E10)</f>
         <v>1</v>
       </c>
       <c r="F11">
@@ -983,22 +1004,14 @@
         <v>744.67450099999996</v>
       </c>
       <c r="G12">
-        <f>1/G2</f>
-        <v>0.81250427888395804</v>
-      </c>
-      <c r="H12">
-        <f>G12*D2/1000</f>
-        <v>0.62809993275701281</v>
+        <f>G2/D2*1000</f>
+        <v>0.6280999327570127</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="G13">
-        <f t="shared" ref="G13:G18" si="4">1/G3</f>
-        <v>6.1270814473216507E-2</v>
-      </c>
-      <c r="H13">
-        <f t="shared" ref="H13:H19" si="5">G13*D3/1000</f>
-        <v>4.5588426967167799E-2</v>
+        <f t="shared" ref="G13:G19" si="4">G3/D3*1000</f>
+        <v>4.5588426967167806E-2</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
@@ -1007,10 +1020,6 @@
       </c>
       <c r="G14">
         <f t="shared" si="4"/>
-        <v>0.16649677845982747</v>
-      </c>
-      <c r="H14">
-        <f t="shared" si="5"/>
         <v>0.12621704533093372</v>
       </c>
     </row>
@@ -1020,10 +1029,6 @@
       </c>
       <c r="G15">
         <f t="shared" si="4"/>
-        <v>1.3319742276786201E-2</v>
-      </c>
-      <c r="H15">
-        <f t="shared" si="5"/>
         <v>1.0284199651391178E-2</v>
       </c>
     </row>
@@ -1033,11 +1038,7 @@
       </c>
       <c r="G16">
         <f t="shared" si="4"/>
-        <v>6.6598711383930986E-3</v>
-      </c>
-      <c r="H16">
-        <f t="shared" si="5"/>
-        <v>3.1940408986176382E-3</v>
+        <v>3.1940408986176386E-3</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
@@ -1046,11 +1047,7 @@
       </c>
       <c r="G17">
         <f t="shared" si="4"/>
-        <v>8.92422732544675E-2</v>
-      </c>
-      <c r="H17">
-        <f t="shared" si="5"/>
-        <v>6.0513043679296309E-2</v>
+        <v>6.0513043679296316E-2</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
@@ -1059,10 +1056,6 @@
       </c>
       <c r="G18">
         <f t="shared" si="4"/>
-        <v>0.18248046919197086</v>
-      </c>
-      <c r="H18">
-        <f t="shared" si="5"/>
         <v>0.12610331071558067</v>
       </c>
     </row>
@@ -1071,10 +1064,7 @@
         <v>15</v>
       </c>
       <c r="G19">
-        <v>0</v>
-      </c>
-      <c r="H19">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
@@ -1082,11 +1072,11 @@
       <c r="A20" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="4">
-        <f>SUM(H12:H19)</f>
+      <c r="G20" s="4">
+        <f>SUM(G12:G19)</f>
         <v>1</v>
       </c>
-      <c r="K20" s="8"/>
+      <c r="K20" s="7"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -1103,12 +1093,8 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G23">
-        <f>1/H2</f>
-        <v>0.60697660439967183</v>
-      </c>
-      <c r="H23">
-        <f>G23*D2/1000</f>
-        <v>0.46921840821833116</v>
+        <f>H2/D2*1000</f>
+        <v>0.46921840821833105</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
@@ -1116,22 +1102,14 @@
         <v>29</v>
       </c>
       <c r="G24">
-        <f t="shared" ref="G24:G30" si="6">1/H3</f>
-        <v>7.9229247034470401E-2</v>
-      </c>
-      <c r="H24">
-        <f t="shared" ref="H24:H30" si="7">G24*D3/1000</f>
-        <v>5.8950362797503639E-2</v>
+        <f t="shared" ref="G24:G30" si="5">H3/D3*1000</f>
+        <v>5.8950362797503646E-2</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B25" s="3"/>
       <c r="G25">
-        <f t="shared" si="6"/>
-        <v>0.25917363860428461</v>
-      </c>
-      <c r="H25">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>0.19647305608494306</v>
       </c>
     </row>
@@ -1143,12 +1121,8 @@
         <v>1</v>
       </c>
       <c r="G26">
-        <f t="shared" si="6"/>
-        <v>2.1485897500873357E-2</v>
-      </c>
-      <c r="H26">
-        <f t="shared" si="7"/>
-        <v>1.6589304432219322E-2</v>
+        <f t="shared" si="5"/>
+        <v>1.6589304432219319E-2</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
@@ -1159,12 +1133,8 @@
         <v>2</v>
       </c>
       <c r="G27">
-        <f t="shared" si="6"/>
-        <v>4.0286057814137508E-3</v>
-      </c>
-      <c r="H27">
-        <f t="shared" si="7"/>
-        <v>1.9320991897371278E-3</v>
+        <f t="shared" si="5"/>
+        <v>1.9320991897371284E-3</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
@@ -1176,22 +1146,14 @@
         <v>3</v>
       </c>
       <c r="G28">
-        <f t="shared" si="6"/>
-        <v>3.4914583438919143E-2</v>
-      </c>
-      <c r="H28">
-        <f t="shared" si="7"/>
+        <f t="shared" si="5"/>
         <v>2.3674741079928539E-2</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G29">
-        <f t="shared" si="6"/>
-        <v>0.32631706829451385</v>
-      </c>
-      <c r="H29">
-        <f t="shared" si="7"/>
-        <v>0.22550173636199211</v>
+        <f t="shared" si="5"/>
+        <v>0.22550173636199214</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
@@ -1199,234 +1161,233 @@
         <v>49</v>
       </c>
       <c r="G30">
+        <f t="shared" si="5"/>
+        <v>7.66029183534512E-3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G31" s="4">
+        <f>SUM(G23:G30)</f>
+        <v>0.99999999999999989</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33" s="8"/>
+      <c r="B33" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="8" cm="1">
+        <f t="array" ref="B34">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-16))</f>
+        <v>0.48554762821834663</v>
+      </c>
+      <c r="C34" s="9">
+        <f>IF(MOD(ROW(),2)=0,B34*$B$27/$B$28,B34*$B$26/$B$28)</f>
+        <v>0.3236984188122311</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A35" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B35" s="8" cm="1">
+        <f t="array" ref="B35">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
+        <v>0.36272553672591512</v>
+      </c>
+      <c r="C35" s="9">
+        <f t="shared" ref="C35:C49" si="6">IF(MOD(ROW(),2)=0,B35*$B$27/$B$28,B35*$B$26/$B$28)</f>
+        <v>0.1209085122419717</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A36" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="8" cm="1">
+        <f t="array" ref="B36">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
+        <v>3.3919977908067271E-2</v>
+      </c>
+      <c r="C36" s="9">
         <f t="shared" si="6"/>
-        <v>1.074294875043667E-2</v>
-      </c>
-      <c r="H30">
-        <f t="shared" si="7"/>
-        <v>7.6602918353451182E-3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="H31" s="4">
-        <f>SUM(H23:H30)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="B33" t="s">
-        <v>50</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>33</v>
-      </c>
-      <c r="B34" cm="1">
-        <f t="array" ref="B34">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-16))</f>
-        <v>1.2307627491803279</v>
-      </c>
-      <c r="C34" s="6">
-        <f>IF(MOD(ROW(),2)=0,B34/$B$27*$B$28,B34/$B$26*$B$28)</f>
-        <v>1.8461441237704919</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" cm="1">
-        <f t="array" ref="B35">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>1.6475099579646018</v>
-      </c>
-      <c r="C35" s="6">
-        <f t="shared" ref="C35:C49" si="8">IF(MOD(ROW(),2)=0,B35/$B$27*$B$28,B35/$B$26*$B$28)</f>
-        <v>4.9425298738938057</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" cm="1">
-        <f t="array" ref="B36">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>16.320984282608695</v>
-      </c>
-      <c r="C36" s="6">
-        <f t="shared" si="8"/>
-        <v>24.481476423913044</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+        <v>2.2613318605378182E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B37" cm="1">
+      <c r="B37" s="8" cm="1">
         <f t="array" ref="B37">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>12.621601711864411</v>
-      </c>
-      <c r="C37" s="6">
-        <f t="shared" si="8"/>
-        <v>37.86480513559323</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+        <v>4.3861899538756993E-2</v>
+      </c>
+      <c r="C37" s="9">
+        <f t="shared" si="6"/>
+        <v>1.4620633179585665E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B38" cm="1">
+      <c r="B38" s="8" cm="1">
         <f t="array" ref="B38">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>6.0061222159999996</v>
-      </c>
-      <c r="C38" s="6">
-        <f t="shared" si="8"/>
-        <v>9.0091833239999985</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+        <v>9.5681986639247596E-2</v>
+      </c>
+      <c r="C38" s="9">
+        <f t="shared" si="6"/>
+        <v>6.3787991092831731E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B39" cm="1">
+      <c r="B39" s="8" cm="1">
         <f t="array" ref="B39">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>3.8584171036269437</v>
-      </c>
-      <c r="C39" s="6">
-        <f t="shared" si="8"/>
-        <v>11.57525131088083</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+        <v>0.14894131199159322</v>
+      </c>
+      <c r="C39" s="9">
+        <f t="shared" si="6"/>
+        <v>4.9647103997197739E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B40" cm="1">
+      <c r="B40" s="8" cm="1">
         <f t="array" ref="B40">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>75.076527699999986</v>
-      </c>
-      <c r="C40" s="6">
-        <f t="shared" si="8"/>
-        <v>112.61479154999998</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+        <v>7.940451119238431E-3</v>
+      </c>
+      <c r="C40" s="9">
+        <f t="shared" si="6"/>
+        <v>5.2936340794922871E-3</v>
+      </c>
+      <c r="D40" s="10"/>
+      <c r="E40" s="11"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B41" cm="1">
+      <c r="B41" s="8" cm="1">
         <f t="array" ref="B41">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>46.542156312499962</v>
-      </c>
-      <c r="C41" s="6">
-        <f t="shared" si="8"/>
-        <v>139.62646893749988</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+        <v>1.28086351307254E-2</v>
+      </c>
+      <c r="C41" s="9">
+        <f t="shared" si="6"/>
+        <v>4.2695450435751335E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B42" cm="1">
+      <c r="B42" s="8" cm="1">
         <f t="array" ref="B42">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>150.1530554</v>
-      </c>
-      <c r="C42" s="6">
-        <f t="shared" si="8"/>
-        <v>225.22958310000001</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+        <v>1.5318460447725265E-3</v>
+      </c>
+      <c r="C42" s="9">
+        <f t="shared" si="6"/>
+        <v>1.0212306965150177E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B43" cm="1">
+      <c r="B43" s="8" cm="1">
         <f t="array" ref="B43">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>248.22483366666665</v>
-      </c>
-      <c r="C43" s="6">
-        <f t="shared" si="8"/>
-        <v>744.67450099999996</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+        <v>9.2662511090197807E-4</v>
+      </c>
+      <c r="C43" s="9">
+        <f t="shared" si="6"/>
+        <v>3.0887503696732602E-4</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B44" cm="1">
+      <c r="B44" s="8" cm="1">
         <f t="array" ref="B44">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>11.205451895522391</v>
-      </c>
-      <c r="C44" s="6">
-        <f t="shared" si="8"/>
-        <v>16.808177843283588</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+        <v>4.1032442605882527E-2</v>
+      </c>
+      <c r="C44" s="9">
+        <f t="shared" si="6"/>
+        <v>2.7354961737255018E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="B45" cm="1">
+      <c r="B45" s="8" cm="1">
         <f t="array" ref="B45">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>28.641326961538486</v>
-      </c>
-      <c r="C45" s="6">
-        <f t="shared" si="8"/>
-        <v>85.92398088461546</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="7" t="s">
+        <v>1.6053273732513623E-2</v>
+      </c>
+      <c r="C45" s="9">
+        <f t="shared" si="6"/>
+        <v>5.3510912441712072E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B46" cm="1">
+      <c r="B46" s="8" cm="1">
         <f t="array" ref="B46">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>5.4800385182481763</v>
-      </c>
-      <c r="C46" s="6">
-        <f t="shared" si="8"/>
-        <v>8.220057777372265</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+        <v>8.7143818973312748E-2</v>
+      </c>
+      <c r="C46" s="9">
+        <f t="shared" si="6"/>
+        <v>5.8095879315541832E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="B47" cm="1">
+      <c r="B47" s="8" cm="1">
         <f t="array" ref="B47">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>3.0645041193415636</v>
-      </c>
-      <c r="C47" s="6">
-        <f t="shared" si="8"/>
-        <v>9.1935123580246909</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+        <v>0.15583320041469104</v>
+      </c>
+      <c r="C47" s="9">
+        <f t="shared" si="6"/>
+        <v>5.1944400138230346E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B48" cm="1">
+      <c r="B48" s="8" cm="1">
         <f t="array" ref="B48">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
         <v>0</v>
       </c>
-      <c r="C48" s="6">
-        <f t="shared" si="8"/>
+      <c r="C48" s="9">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="A49" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B49" cm="1">
+      <c r="B49" s="8" cm="1">
         <f t="array" ref="B49">IF(MOD(ROW(),2)=0, INDEX(G:G, ROW()/2-15), INDEX(H:H, ROW()/2-15))</f>
-        <v>93.084312624999995</v>
-      </c>
-      <c r="C49" s="6">
-        <f t="shared" si="8"/>
-        <v>279.25293787499999</v>
+        <v>5.4621940740683435E-3</v>
+      </c>
+      <c r="C49" s="9">
+        <f t="shared" si="6"/>
+        <v>1.8207313580227813E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>